<commit_message>
easi: activate easi-screening v2, pinned (D20); calculator 1.1 from v2; StreamCurves' vendored EASI re-synced
export_easi_method.py --write-easi-data --pin: the two method files v2 changes
(screening-methods.json, scoring-identity.json) and data/source/adopted-method.json, the pin EASI
loads its adopted method by (cache, then the library release, then this bundled copy, each
verified against the pin; never a newer version). The committed workbook regenerated from the v2
files is byte-identical to the library's (8da078bf).
</commit_message>
<xml_diff>
--- a/apps/easi/www/calculator/EASI_Calculator_1.1.xlsx
+++ b/apps/easi/www/calculator/EASI_Calculator_1.1.xlsx
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>EASI calculator v1.1, scoring method 0ab411ad0326 (Alternative 2: NARS-9 references)</t>
+          <t>EASI calculator v1.1, scoring method e91118cc821c (Alternative 2 with corrected cross-section quality checks (E5b))</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -17725,7 +17725,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>0ab411ad0326</t>
+          <t>e91118cc821c</t>
         </is>
       </c>
     </row>
@@ -17737,7 +17737,7 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>alternative-2 (Alternative 2: NARS-9 references)</t>
+          <t>alternative-2-e5b (Alternative 2 with corrected cross-section quality checks (E5b))</t>
         </is>
       </c>
     </row>
@@ -17773,7 +17773,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>78c1e2921198905ee6e53f18147e2aa33f9a6ffd87ff3e7a23844238b3fb73f3</t>
+          <t>e754bf570291e0231d11e127e594a7fa375b3f227ee2f0d6591c45f9faa4ac49</t>
         </is>
       </c>
     </row>

</xml_diff>